<commit_message>
feat: plantilla de excel con 10 filas de ejemplo en vez de 3
</commit_message>
<xml_diff>
--- a/public/plantilla-pedidos.xlsx
+++ b/public/plantilla-pedidos.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -583,6 +583,216 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Equipos de computo</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Maria Fernandez Soto</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>998877665</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Calle Los Alamos 234, La Molina</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Ropa y calzado</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Jorge Paredes Rios</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>911223344</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Av. Angamos 567, Surquillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Muebles pequenos</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Patricia Salas Nunez</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>944556677</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Jr. Camana 890, Cercado de Lima</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Insumos medicos</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Roberto Diaz Campos</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>977889900</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Av. Brasil 456, Pueblo Libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Material de oficina</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Claudia Herrera Luna</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>933221100</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Av. Salaverry 321, Jesus Maria</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Alimentos no perecibles</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Fernando Castro Gil</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>966554433</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Calle Las Begonias 111, San Isidro</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Juguetes</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Andrea Morales Quispe</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>922334455</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Av. La Marina 678, San Miguel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>